<commit_message>
updated code to include structures A3 and A4
</commit_message>
<xml_diff>
--- a/verification_burde/associators_results.xlsx
+++ b/verification_burde/associators_results.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josemarialoza/capstone/verification_burde/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E581E40D-BA8A-3849-A695-4CA3B3FAF8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8224F576-8E91-6741-A6F6-52A7F527080D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="860" windowWidth="27640" windowHeight="16700" xr2:uid="{649C684C-B9D2-864E-BB41-4ED8492614DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="128">
   <si>
     <t>LSS 2</t>
   </si>
@@ -355,12 +355,99 @@
   <si>
     <t xml:space="preserve">3u(-uv + v^2 + 1)E + 3vF + (- 6v^2)H = 0 </t>
   </si>
+  <si>
+    <t>LSS 3</t>
+  </si>
+  <si>
+    <t>LSS 4</t>
+  </si>
+  <si>
+    <t>-F</t>
+  </si>
+  <si>
+    <t>-F + H</t>
+  </si>
+  <si>
+    <t>2H</t>
+  </si>
+  <si>
+    <t>-H</t>
+  </si>
+  <si>
+    <t>-E + 2H</t>
+  </si>
+  <si>
+    <t>-E - H</t>
+  </si>
+  <si>
+    <t>-3H</t>
+  </si>
+  <si>
+    <t>-2E</t>
+  </si>
+  <si>
+    <t>-E  - H</t>
+  </si>
+  <si>
+    <t>b(1-b)E</t>
+  </si>
+  <si>
+    <t>(-b^2 - 3b + 2)E = 0</t>
+  </si>
+  <si>
+    <t>(b^2 - 1)E</t>
+  </si>
+  <si>
+    <t>(1 - 3b)E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(b^2 - 3b - 2)F = 0 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(b^2 - 1)F </t>
+  </si>
+  <si>
+    <t>(3b + 1)F</t>
+  </si>
+  <si>
+    <t>(1 - b)H</t>
+  </si>
+  <si>
+    <t>(b^2  + 3b - 2)E = 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-b^2 + 3b + 2)F = 0 </t>
+  </si>
+  <si>
+    <t>-b(b + 1)F</t>
+  </si>
+  <si>
+    <t>-2H</t>
+  </si>
+  <si>
+    <t>(b + 1)H</t>
+  </si>
+  <si>
+    <t>-3E</t>
+  </si>
+  <si>
+    <t>2E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3E </t>
+  </si>
+  <si>
+    <t>(b - 1)E</t>
+  </si>
+  <si>
+    <t>-(b + 1)F</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -381,8 +468,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -401,8 +495,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -462,11 +568,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -489,6 +604,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -824,7 +954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF4F6DDB-020B-D943-B081-176EC956BF99}">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="47.1640625" customWidth="1"/>
@@ -1783,10 +1913,948 @@
         <v>83</v>
       </c>
     </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="11">
+        <v>0</v>
+      </c>
+      <c r="D59" s="11">
+        <v>0</v>
+      </c>
+      <c r="E59" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C61" s="11">
+        <v>0</v>
+      </c>
+      <c r="D61" s="11">
+        <v>0</v>
+      </c>
+      <c r="E61" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E62" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" s="11">
+        <v>0</v>
+      </c>
+      <c r="D63" s="11">
+        <v>0</v>
+      </c>
+      <c r="E63" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C64" s="11">
+        <v>0</v>
+      </c>
+      <c r="D64" s="11">
+        <v>0</v>
+      </c>
+      <c r="E64" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="11">
+        <v>0</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C66" s="11">
+        <v>0</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="E66" s="12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C67" s="11">
+        <v>0</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="E67" s="12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C68" s="11">
+        <v>0</v>
+      </c>
+      <c r="D68" s="11">
+        <v>0</v>
+      </c>
+      <c r="E68" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" s="11">
+        <v>0</v>
+      </c>
+      <c r="D69" s="11">
+        <v>0</v>
+      </c>
+      <c r="E69" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C70" s="11">
+        <v>0</v>
+      </c>
+      <c r="D70" s="11">
+        <v>0</v>
+      </c>
+      <c r="E70" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C71" s="11">
+        <v>0</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C72" s="11">
+        <v>0</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C73" s="11">
+        <v>0</v>
+      </c>
+      <c r="D73" s="11">
+        <v>0</v>
+      </c>
+      <c r="E73" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C74" s="11">
+        <v>0</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E74" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C75" s="11">
+        <v>0</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E75" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C76" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D76" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="E76" s="12" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C77" s="11">
+        <v>0</v>
+      </c>
+      <c r="D77" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E77" s="12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78" s="11">
+        <v>0</v>
+      </c>
+      <c r="D78" s="11">
+        <v>0</v>
+      </c>
+      <c r="E78" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C79" s="11">
+        <v>0</v>
+      </c>
+      <c r="D79" s="11">
+        <v>0</v>
+      </c>
+      <c r="E79" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80" s="11">
+        <v>0</v>
+      </c>
+      <c r="D80" s="11">
+        <v>0</v>
+      </c>
+      <c r="E80" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" s="12">
+        <v>0</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E81" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C82" s="11">
+        <v>0</v>
+      </c>
+      <c r="D82" s="11">
+        <v>0</v>
+      </c>
+      <c r="E82" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C83" s="11">
+        <v>0</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E83" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C84" s="11">
+        <v>0</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E84" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E85" s="12" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="10"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="11">
+        <v>0</v>
+      </c>
+      <c r="D87" s="11">
+        <v>0</v>
+      </c>
+      <c r="E87" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" s="11">
+        <v>0</v>
+      </c>
+      <c r="D88" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E88" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C89" s="11">
+        <v>0</v>
+      </c>
+      <c r="D89" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E89" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90" s="11">
+        <v>0</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E90" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91" s="11">
+        <v>0</v>
+      </c>
+      <c r="D91" s="11">
+        <v>0</v>
+      </c>
+      <c r="E91" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C92" s="11">
+        <v>0</v>
+      </c>
+      <c r="D92" s="11">
+        <v>0</v>
+      </c>
+      <c r="E92" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D93" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E93" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C94" s="11">
+        <v>0</v>
+      </c>
+      <c r="D94" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C95" s="11">
+        <v>0</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="E95" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C96" s="11">
+        <v>0</v>
+      </c>
+      <c r="D96" s="11">
+        <v>0</v>
+      </c>
+      <c r="E96" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C97" s="11">
+        <v>0</v>
+      </c>
+      <c r="D97" s="11">
+        <v>0</v>
+      </c>
+      <c r="E97" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C98" s="11">
+        <v>0</v>
+      </c>
+      <c r="D98" s="11">
+        <v>0</v>
+      </c>
+      <c r="E98" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C99" s="11">
+        <v>0</v>
+      </c>
+      <c r="D99" s="11">
+        <v>0</v>
+      </c>
+      <c r="E99" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C100" s="11">
+        <v>0</v>
+      </c>
+      <c r="D100" s="11">
+        <v>0</v>
+      </c>
+      <c r="E100" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C101" s="11">
+        <v>0</v>
+      </c>
+      <c r="D101" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E101" s="11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D102" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E102" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C103" s="11">
+        <v>0</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="E103" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A104" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C104" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D104" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E104" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C105" s="11">
+        <v>0</v>
+      </c>
+      <c r="D105" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E105" s="12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C106" s="11">
+        <v>0</v>
+      </c>
+      <c r="D106" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E106" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C107" s="11">
+        <v>0</v>
+      </c>
+      <c r="D107" s="11">
+        <v>0</v>
+      </c>
+      <c r="E107" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C108" s="11">
+        <v>0</v>
+      </c>
+      <c r="D108" s="11">
+        <v>0</v>
+      </c>
+      <c r="E108" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C109" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D109" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E109" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C110" s="1">
+        <v>0</v>
+      </c>
+      <c r="D110" s="1">
+        <v>0</v>
+      </c>
+      <c r="E110" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C111" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="D111" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E111" s="11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C112" s="1">
+        <v>0</v>
+      </c>
+      <c r="D112" s="1">
+        <v>0</v>
+      </c>
+      <c r="E112" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D113" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E113" s="11" t="s">
+        <v>124</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A86:E86"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>